<commit_message>
#7 Changes Completed and Fresh Deliverables Generated
</commit_message>
<xml_diff>
--- a/Design-Files-v2.4/Control-Board_v2.4/Deliverables/BOM/Control-Board_v2.4.xlsx
+++ b/Design-Files-v2.4/Control-Board_v2.4/Deliverables/BOM/Control-Board_v2.4.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eSpark Cons Group\Documents\GitHub\Melih-SoundSensor\bradfairman-ledproject\Design-Files\Button-Board_v2.4\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eSpark Cons Group\Documents\GitHub\Melih-SoundSensor\bradfairman-ledproject\Design-Files-v2.4\Control-Board_v2.4\Project Outputs for Control-Board_v2.4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{653734CA-9200-4BC6-92C3-F7E6A0550B8B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6234415-B42F-4E55-B028-4539071276CF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="194">
   <si>
     <t>#</t>
   </si>
@@ -55,9 +55,6 @@
     <t>Resistor</t>
   </si>
   <si>
-    <t>[NoParam], Resistor</t>
-  </si>
-  <si>
     <t>Resistors</t>
   </si>
   <si>
@@ -274,7 +271,7 @@
     <t>RES 100K OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t>No Gull Wing 50mA 100MΩ 80000 260gf@±50gf 12V -25℃~+85℃ 1.7mm Golden Round Button Brick nogging SPST SMD Tactile Switches ROHS</t>
+    <t>Tactile Switches 5.20 x 5.20 Tact Switch for SMT</t>
   </si>
   <si>
     <t>IC Pb On/off Controller TSOT23-8</t>
@@ -349,7 +346,7 @@
     <t>Res-1206</t>
   </si>
   <si>
-    <t>TC-0522C-1.7-260G_</t>
+    <t>PTS526SP15SMTR2 LFS</t>
   </si>
   <si>
     <t>TSOT-23-8</t>
@@ -460,7 +457,7 @@
     <t>RC0402FR-07100KL</t>
   </si>
   <si>
-    <t>TC-0522C-1.7-260G</t>
+    <t>PTS526SP15SMTR2LFS</t>
   </si>
   <si>
     <t>LTC2950ITS8-2#TRPBF</t>
@@ -529,7 +526,7 @@
     <t>YAGEO</t>
   </si>
   <si>
-    <t>HCTL</t>
+    <t>ITT C&amp;K</t>
   </si>
   <si>
     <t>Analog Devices / Linear Technology</t>
@@ -602,6 +599,9 @@
   </si>
   <si>
     <t>Quantity</t>
+  </si>
+  <si>
+    <t>Connector</t>
   </si>
 </sst>
 </file>
@@ -1129,25 +1129,25 @@
         <v>1</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1160,22 +1160,22 @@
         <v>2</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="J3" s="7">
         <v>1</v>
@@ -1191,22 +1191,22 @@
         <v>2</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="J4" s="9">
         <v>1</v>
@@ -1222,22 +1222,22 @@
         <v>2</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J5" s="7">
         <v>2</v>
@@ -1253,22 +1253,22 @@
         <v>2</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J6" s="9">
         <v>4</v>
@@ -1284,22 +1284,22 @@
         <v>3</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="J7" s="7">
         <v>2</v>
@@ -1315,22 +1315,22 @@
         <v>2</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="J8" s="9">
         <v>2</v>
@@ -1346,22 +1346,22 @@
         <v>2</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -1377,22 +1377,22 @@
         <v>4</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J10" s="9">
         <v>1</v>
@@ -1408,22 +1408,22 @@
         <v>4</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J11" s="7">
         <v>1</v>
@@ -1435,24 +1435,26 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C12" s="13"/>
+      <c r="C12" s="13" t="s">
+        <v>193</v>
+      </c>
       <c r="D12" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
@@ -1468,20 +1470,20 @@
         <v>5</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H13" s="7"/>
       <c r="I13" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J13" s="7">
         <v>1</v>
@@ -1497,22 +1499,22 @@
         <v>6</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -1528,22 +1530,22 @@
         <v>6</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
@@ -1559,22 +1561,22 @@
         <v>7</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="J16" s="9">
         <v>3</v>
@@ -1590,22 +1592,22 @@
         <v>8</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
@@ -1621,22 +1623,22 @@
         <v>9</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="J18" s="9">
         <v>3</v>
@@ -1652,22 +1654,22 @@
         <v>8</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J19" s="7">
         <v>1</v>
@@ -1681,22 +1683,22 @@
       </c>
       <c r="C20" s="13"/>
       <c r="D20" s="9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
@@ -1712,22 +1714,22 @@
         <v>10</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="J21" s="7">
         <v>3</v>
@@ -1740,25 +1742,25 @@
         <v>20</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J22" s="9">
         <v>3</v>
@@ -1774,22 +1776,22 @@
         <v>10</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="J23" s="7">
         <v>3</v>
@@ -1805,22 +1807,22 @@
         <v>10</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="J24" s="9">
         <v>10</v>
@@ -1836,22 +1838,22 @@
         <v>10</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J25" s="7">
         <v>1</v>
@@ -1867,22 +1869,22 @@
         <v>10</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="J26" s="9">
         <v>3</v>
@@ -1895,25 +1897,25 @@
         <v>25</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
@@ -1929,22 +1931,22 @@
         <v>10</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="J28" s="9">
         <v>1</v>
@@ -1960,22 +1962,22 @@
         <v>10</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
@@ -1991,22 +1993,22 @@
         <v>10</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="J30" s="9">
         <v>2</v>
@@ -2022,53 +2024,53 @@
         <v>10</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="J31" s="7">
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="11">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>
@@ -2081,25 +2083,25 @@
         <v>31</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
@@ -2112,25 +2114,25 @@
         <v>32</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
@@ -2143,25 +2145,25 @@
         <v>33</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J35" s="7">
         <v>1</v>
@@ -2174,25 +2176,25 @@
         <v>34</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I36" s="10" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J36" s="9">
         <v>1</v>
@@ -2205,25 +2207,25 @@
         <v>35</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H37" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="J37" s="7">
         <v>1</v>
@@ -2236,25 +2238,25 @@
         <v>36</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I38" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="J38" s="9">
         <v>1</v>
@@ -2267,25 +2269,25 @@
         <v>37</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="H39" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="I39" s="8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J39" s="7">
         <v>1</v>

</xml_diff>